<commit_message>
build: register comet-pcr (PCR Method/CarbonSig ext) namespace in ontology map + rebuild docs
</commit_message>
<xml_diff>
--- a/docs/comet-ontology-values.xlsx
+++ b/docs/comet-ontology-values.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Terms'!$A$1:$N$947</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Namespaces'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Namespaces'!$A$1:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Alignments'!$A$1:$G$368</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Schema Fields'!$A$1:$H$81</definedName>
   </definedNames>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11">
@@ -54026,7 +54026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -54372,38 +54372,42 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>cadtrust</t>
+          <t>comet-pcr</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>CAD Trust Data Dictionary</t>
+          <t>PCR Method / CarbonSig (ext)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>CAD Trust (incorporated)</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
+          <t>Extension</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>https://comet.carbon/ext/pcr#</t>
+        </is>
+      </c>
       <c r="E12" s="4" t="n">
-        <v>246</v>
+        <v>0</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>#5a5a5a</t>
+          <t>#0a7c5a</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>cadpick</t>
+          <t>cadtrust</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CAD Trust Picklist Values</t>
+          <t>CAD Trust Data Dictionary</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -54413,16 +54417,42 @@
       </c>
       <c r="D13" s="4" t="inlineStr"/>
       <c r="E13" s="4" t="n">
+        <v>246</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>#5a5a5a</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>cadpick</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>CAD Trust Picklist Values</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>CAD Trust (incorporated)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="n">
         <v>403</v>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>#8a8a8a</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F13"/>
+  <autoFilter ref="A1:F14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>